<commit_message>
small-tender: exclude non-goods from auction report and trace exclusions
</commit_message>
<xml_diff>
--- a/exports/small_tender_report_auction_prod.xlsx
+++ b/exports/small_tender_report_auction_prod.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q10"/>
+  <dimension ref="A1:R6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -484,20 +484,25 @@
       </c>
       <c r="N1" t="inlineStr">
         <is>
+          <t>found_offer_unit_price</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
           <t>margin_pct</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>decision_status</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>risk_level</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>decision_reason</t>
         </is>
@@ -506,20 +511,20 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>10208354</t>
+          <t>10208353</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Монтаж сетки защитной  в спортивных залах, м2</t>
+          <t>Стенд ProfMarker Гражданская оборона ГО и ЧС 100х75 см</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>388</v>
+        <v>2790</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>https://zakupki.mos.ru/auction/10208354</t>
+          <t>https://zakupki.mos.ru/auction/10208353</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -535,36 +540,36 @@
       <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr">
         <is>
-          <t>exports/tz_files_auction/10208354/ТЗ монтаж сетки (2).docx</t>
+          <t>exports/tz_files_auction/10208353/Техническое задание.docx</t>
         </is>
       </c>
       <c r="J2" t="n">
-        <v>6681</v>
+        <v>18272</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>full</t>
+          <t>none</t>
         </is>
       </c>
       <c r="L2" t="n">
-        <v>0.0048</v>
+        <v>0.0065</v>
       </c>
       <c r="M2" t="b">
         <v>0</v>
       </c>
-      <c r="O2" t="inlineStr">
+      <c r="P2" t="inlineStr">
         <is>
           <t>reject</t>
         </is>
       </c>
-      <c r="P2" t="inlineStr">
+      <c r="Q2" t="inlineStr">
         <is>
           <t>critical</t>
         </is>
       </c>
-      <c r="Q2" t="inlineStr">
-        <is>
-          <t>missing_price_for_margin</t>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>strict_full_match_required:none</t>
         </is>
       </c>
     </row>
@@ -576,7 +581,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Стенд ProfMarker Гражданская оборона ГО и ЧС 100х75 см</t>
+          <t>Стенд информационный   ProfMarker " "Пожарная безопасность" , красный, 900х740 мм., 1 карман А4</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -612,22 +617,22 @@
         </is>
       </c>
       <c r="L3" t="n">
-        <v>0.0065</v>
+        <v>0.0104</v>
       </c>
       <c r="M3" t="b">
         <v>0</v>
       </c>
-      <c r="O3" t="inlineStr">
+      <c r="P3" t="inlineStr">
         <is>
           <t>reject</t>
         </is>
       </c>
-      <c r="P3" t="inlineStr">
+      <c r="Q3" t="inlineStr">
         <is>
           <t>critical</t>
         </is>
       </c>
-      <c r="Q3" t="inlineStr">
+      <c r="R3" t="inlineStr">
         <is>
           <t>strict_full_match_required:none</t>
         </is>
@@ -641,7 +646,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Стенд информационный   ProfMarker " "Пожарная безопасность" , красный, 900х740 мм., 1 карман А4</t>
+          <t>Стенд информационный  "ПолиЦентр" "Воинский Учет" 740х780 мм с 6 карманами А4</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -677,22 +682,22 @@
         </is>
       </c>
       <c r="L4" t="n">
-        <v>0.0104</v>
+        <v>0.0091</v>
       </c>
       <c r="M4" t="b">
         <v>0</v>
       </c>
-      <c r="O4" t="inlineStr">
+      <c r="P4" t="inlineStr">
         <is>
           <t>reject</t>
         </is>
       </c>
-      <c r="P4" t="inlineStr">
+      <c r="Q4" t="inlineStr">
         <is>
           <t>critical</t>
         </is>
       </c>
-      <c r="Q4" t="inlineStr">
+      <c r="R4" t="inlineStr">
         <is>
           <t>strict_full_match_required:none</t>
         </is>
@@ -701,20 +706,20 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>10208353</t>
+          <t>10208351</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Стенд информационный  "ПолиЦентр" "Воинский Учет" 740х780 мм с 6 карманами А4</t>
+          <t>Зажим прокалывающий "Тайко Электроникс РУС" Al/Cu 10-50 мм2 / Al/Cu 1.5-10 мм2</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>2790</v>
+        <v>320</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>https://zakupki.mos.ru/auction/10208353</t>
+          <t>https://zakupki.mos.ru/auction/10208351</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -730,11 +735,11 @@
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr">
         <is>
-          <t>exports/tz_files_auction/10208353/Техническое задание.docx</t>
+          <t>exports/tz_files_auction/10208351/Приложение №1 к Договору (Техническое задание).docx</t>
         </is>
       </c>
       <c r="J5" t="n">
-        <v>18272</v>
+        <v>13281</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
@@ -742,22 +747,22 @@
         </is>
       </c>
       <c r="L5" t="n">
-        <v>0.0091</v>
+        <v>0.0059</v>
       </c>
       <c r="M5" t="b">
         <v>0</v>
       </c>
-      <c r="O5" t="inlineStr">
+      <c r="P5" t="inlineStr">
         <is>
           <t>reject</t>
         </is>
       </c>
-      <c r="P5" t="inlineStr">
+      <c r="Q5" t="inlineStr">
         <is>
           <t>critical</t>
         </is>
       </c>
-      <c r="Q5" t="inlineStr">
+      <c r="R5" t="inlineStr">
         <is>
           <t>strict_full_match_required:none</t>
         </is>
@@ -766,20 +771,20 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>10208336</t>
+          <t>10208351</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Ремонт электрооборудования</t>
+          <t>Колодка клеммная EKF plc-jxb-10/35gy JXB-10/3 серая 70А 50 шт</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>25417.81</v>
+        <v>320</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>https://zakupki.mos.ru/auction/10208336</t>
+          <t>https://zakupki.mos.ru/auction/10208351</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -795,11 +800,11 @@
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr">
         <is>
-          <t>exports/tz_files_auction/10208336/Техзадание.docx</t>
+          <t>exports/tz_files_auction/10208351/Приложение №1 к Договору (Техническое задание).docx</t>
         </is>
       </c>
       <c r="J6" t="n">
-        <v>3056</v>
+        <v>13281</v>
       </c>
       <c r="K6" t="inlineStr">
         <is>
@@ -807,282 +812,22 @@
         </is>
       </c>
       <c r="L6" t="n">
-        <v>0.0095</v>
+        <v>0</v>
       </c>
       <c r="M6" t="b">
         <v>0</v>
       </c>
-      <c r="O6" t="inlineStr">
+      <c r="P6" t="inlineStr">
         <is>
           <t>reject</t>
         </is>
       </c>
-      <c r="P6" t="inlineStr">
+      <c r="Q6" t="inlineStr">
         <is>
           <t>critical</t>
         </is>
       </c>
-      <c r="Q6" t="inlineStr">
-        <is>
-          <t>strict_full_match_required:none</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>10208352</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Демонтаж оборудования охранной системы видеонаблюдения</t>
-        </is>
-      </c>
-      <c r="C7" t="n">
-        <v>2102.8</v>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>https://zakupki.mos.ru/auction/10208352</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>2026-05-22T07:27:55.695031+00:00</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>exports/tz_files_auction/10208352/Приложение 1 к Контракту №____ТЗ (демонтаж, монтаж видеокамер).docx</t>
-        </is>
-      </c>
-      <c r="J7" t="n">
-        <v>28010</v>
-      </c>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="L7" t="n">
-        <v>0.0054</v>
-      </c>
-      <c r="M7" t="b">
-        <v>0</v>
-      </c>
-      <c r="O7" t="inlineStr">
-        <is>
-          <t>reject</t>
-        </is>
-      </c>
-      <c r="P7" t="inlineStr">
-        <is>
-          <t>critical</t>
-        </is>
-      </c>
-      <c r="Q7" t="inlineStr">
-        <is>
-          <t>strict_full_match_required:none</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>10208352</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Монтаж оборудования охранной системы видеонаблюдения</t>
-        </is>
-      </c>
-      <c r="C8" t="n">
-        <v>2102.8</v>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>https://zakupki.mos.ru/auction/10208352</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>2026-05-22T07:27:55.695031+00:00</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>exports/tz_files_auction/10208352/Приложение 1 к Контракту №____ТЗ (демонтаж, монтаж видеокамер).docx</t>
-        </is>
-      </c>
-      <c r="J8" t="n">
-        <v>28010</v>
-      </c>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="L8" t="n">
-        <v>0.0054</v>
-      </c>
-      <c r="M8" t="b">
-        <v>0</v>
-      </c>
-      <c r="O8" t="inlineStr">
-        <is>
-          <t>reject</t>
-        </is>
-      </c>
-      <c r="P8" t="inlineStr">
-        <is>
-          <t>critical</t>
-        </is>
-      </c>
-      <c r="Q8" t="inlineStr">
-        <is>
-          <t>strict_full_match_required:none</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>10208351</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Зажим прокалывающий "Тайко Электроникс РУС" Al/Cu 10-50 мм2 / Al/Cu 1.5-10 мм2</t>
-        </is>
-      </c>
-      <c r="C9" t="n">
-        <v>320</v>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>https://zakupki.mos.ru/auction/10208351</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>2026-05-22T07:27:55.695031+00:00</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>exports/tz_files_auction/10208351/Приложение №1 к Договору (Техническое задание).docx</t>
-        </is>
-      </c>
-      <c r="J9" t="n">
-        <v>13281</v>
-      </c>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="L9" t="n">
-        <v>0.0059</v>
-      </c>
-      <c r="M9" t="b">
-        <v>0</v>
-      </c>
-      <c r="O9" t="inlineStr">
-        <is>
-          <t>reject</t>
-        </is>
-      </c>
-      <c r="P9" t="inlineStr">
-        <is>
-          <t>critical</t>
-        </is>
-      </c>
-      <c r="Q9" t="inlineStr">
-        <is>
-          <t>strict_full_match_required:none</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>10208351</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Колодка клеммная EKF plc-jxb-10/35gy JXB-10/3 серая 70А 50 шт</t>
-        </is>
-      </c>
-      <c r="C10" t="n">
-        <v>320</v>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>https://zakupki.mos.ru/auction/10208351</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>2026-05-22T07:27:55.695031+00:00</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr"/>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>exports/tz_files_auction/10208351/Приложение №1 к Договору (Техническое задание).docx</t>
-        </is>
-      </c>
-      <c r="J10" t="n">
-        <v>13281</v>
-      </c>
-      <c r="K10" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="L10" t="n">
-        <v>0</v>
-      </c>
-      <c r="M10" t="b">
-        <v>0</v>
-      </c>
-      <c r="O10" t="inlineStr">
-        <is>
-          <t>reject</t>
-        </is>
-      </c>
-      <c r="P10" t="inlineStr">
-        <is>
-          <t>critical</t>
-        </is>
-      </c>
-      <c r="Q10" t="inlineStr">
+      <c r="R6" t="inlineStr">
         <is>
           <t>strict_full_match_required:none</t>
         </is>

</xml_diff>

<commit_message>
small-tender: resolve auction prices from offer_source_url fallback
</commit_message>
<xml_diff>
--- a/exports/small_tender_report_auction_prod.xlsx
+++ b/exports/small_tender_report_auction_prod.xlsx
@@ -527,6 +527,9 @@
           <t>https://zakupki.mos.ru/auction/10208353</t>
         </is>
       </c>
+      <c r="E2" t="n">
+        <v>3485</v>
+      </c>
       <c r="F2" t="inlineStr">
         <is>
           <t>2026-05-22T07:27:55.695031+00:00</t>
@@ -556,6 +559,12 @@
       </c>
       <c r="M2" t="b">
         <v>0</v>
+      </c>
+      <c r="N2" t="n">
+        <v>3485</v>
+      </c>
+      <c r="O2" t="n">
+        <v>-24.91</v>
       </c>
       <c r="P2" t="inlineStr">
         <is>
@@ -592,6 +601,9 @@
           <t>https://zakupki.mos.ru/auction/10208353</t>
         </is>
       </c>
+      <c r="E3" t="n">
+        <v>2985</v>
+      </c>
       <c r="F3" t="inlineStr">
         <is>
           <t>2026-05-22T07:27:55.695031+00:00</t>
@@ -621,6 +633,12 @@
       </c>
       <c r="M3" t="b">
         <v>0</v>
+      </c>
+      <c r="N3" t="n">
+        <v>2985</v>
+      </c>
+      <c r="O3" t="n">
+        <v>-6.99</v>
       </c>
       <c r="P3" t="inlineStr">
         <is>
@@ -657,6 +675,9 @@
           <t>https://zakupki.mos.ru/auction/10208353</t>
         </is>
       </c>
+      <c r="E4" t="n">
+        <v>2790</v>
+      </c>
       <c r="F4" t="inlineStr">
         <is>
           <t>2026-05-22T07:27:55.695031+00:00</t>
@@ -685,6 +706,12 @@
         <v>0.0091</v>
       </c>
       <c r="M4" t="b">
+        <v>0</v>
+      </c>
+      <c r="N4" t="n">
+        <v>2790</v>
+      </c>
+      <c r="O4" t="n">
         <v>0</v>
       </c>
       <c r="P4" t="inlineStr">
@@ -722,6 +749,9 @@
           <t>https://zakupki.mos.ru/auction/10208351</t>
         </is>
       </c>
+      <c r="E5" t="n">
+        <v>320</v>
+      </c>
       <c r="F5" t="inlineStr">
         <is>
           <t>2026-05-22T07:27:55.695031+00:00</t>
@@ -750,6 +780,12 @@
         <v>0.0059</v>
       </c>
       <c r="M5" t="b">
+        <v>0</v>
+      </c>
+      <c r="N5" t="n">
+        <v>320</v>
+      </c>
+      <c r="O5" t="n">
         <v>0</v>
       </c>
       <c r="P5" t="inlineStr">
@@ -787,6 +823,9 @@
           <t>https://zakupki.mos.ru/auction/10208351</t>
         </is>
       </c>
+      <c r="E6" t="n">
+        <v>3500</v>
+      </c>
       <c r="F6" t="inlineStr">
         <is>
           <t>2026-05-22T07:27:55.695031+00:00</t>
@@ -816,6 +855,12 @@
       </c>
       <c r="M6" t="b">
         <v>0</v>
+      </c>
+      <c r="N6" t="n">
+        <v>3500</v>
+      </c>
+      <c r="O6" t="n">
+        <v>-993.75</v>
       </c>
       <c r="P6" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
small-tender: expose explicit market price source fields in auction report
</commit_message>
<xml_diff>
--- a/exports/small_tender_report_auction_prod.xlsx
+++ b/exports/small_tender_report_auction_prod.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R6"/>
+  <dimension ref="A1:U6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -489,20 +489,35 @@
       </c>
       <c r="O1" t="inlineStr">
         <is>
+          <t>market_price_source_url</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>market_price_source_domain</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>market_price_source_note</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
           <t>margin_pct</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>decision_status</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>risk_level</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>decision_reason</t>
         </is>
@@ -563,20 +578,35 @@
       <c r="N2" t="n">
         <v>3485</v>
       </c>
-      <c r="O2" t="n">
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>https://zakupki.mos.ru/auction/10208353</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>zakupki.mos.ru</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>auction_api_costPerUnit</t>
+        </is>
+      </c>
+      <c r="R2" t="n">
         <v>-24.91</v>
       </c>
-      <c r="P2" t="inlineStr">
+      <c r="S2" t="inlineStr">
         <is>
           <t>reject</t>
         </is>
       </c>
-      <c r="Q2" t="inlineStr">
+      <c r="T2" t="inlineStr">
         <is>
           <t>critical</t>
         </is>
       </c>
-      <c r="R2" t="inlineStr">
+      <c r="U2" t="inlineStr">
         <is>
           <t>strict_full_match_required:none</t>
         </is>
@@ -637,20 +667,35 @@
       <c r="N3" t="n">
         <v>2985</v>
       </c>
-      <c r="O3" t="n">
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>https://zakupki.mos.ru/auction/10208353</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>zakupki.mos.ru</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>auction_api_costPerUnit</t>
+        </is>
+      </c>
+      <c r="R3" t="n">
         <v>-6.99</v>
       </c>
-      <c r="P3" t="inlineStr">
+      <c r="S3" t="inlineStr">
         <is>
           <t>reject</t>
         </is>
       </c>
-      <c r="Q3" t="inlineStr">
+      <c r="T3" t="inlineStr">
         <is>
           <t>critical</t>
         </is>
       </c>
-      <c r="R3" t="inlineStr">
+      <c r="U3" t="inlineStr">
         <is>
           <t>strict_full_match_required:none</t>
         </is>
@@ -711,20 +756,35 @@
       <c r="N4" t="n">
         <v>2790</v>
       </c>
-      <c r="O4" t="n">
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>https://zakupki.mos.ru/auction/10208353</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>zakupki.mos.ru</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>auction_api_costPerUnit</t>
+        </is>
+      </c>
+      <c r="R4" t="n">
         <v>0</v>
       </c>
-      <c r="P4" t="inlineStr">
+      <c r="S4" t="inlineStr">
         <is>
           <t>reject</t>
         </is>
       </c>
-      <c r="Q4" t="inlineStr">
+      <c r="T4" t="inlineStr">
         <is>
           <t>critical</t>
         </is>
       </c>
-      <c r="R4" t="inlineStr">
+      <c r="U4" t="inlineStr">
         <is>
           <t>strict_full_match_required:none</t>
         </is>
@@ -785,20 +845,35 @@
       <c r="N5" t="n">
         <v>320</v>
       </c>
-      <c r="O5" t="n">
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>https://zakupki.mos.ru/auction/10208351</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>zakupki.mos.ru</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>auction_api_costPerUnit</t>
+        </is>
+      </c>
+      <c r="R5" t="n">
         <v>0</v>
       </c>
-      <c r="P5" t="inlineStr">
+      <c r="S5" t="inlineStr">
         <is>
           <t>reject</t>
         </is>
       </c>
-      <c r="Q5" t="inlineStr">
+      <c r="T5" t="inlineStr">
         <is>
           <t>critical</t>
         </is>
       </c>
-      <c r="R5" t="inlineStr">
+      <c r="U5" t="inlineStr">
         <is>
           <t>strict_full_match_required:none</t>
         </is>
@@ -859,20 +934,35 @@
       <c r="N6" t="n">
         <v>3500</v>
       </c>
-      <c r="O6" t="n">
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>https://zakupki.mos.ru/auction/10208351</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>zakupki.mos.ru</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>auction_api_costPerUnit</t>
+        </is>
+      </c>
+      <c r="R6" t="n">
         <v>-993.75</v>
       </c>
-      <c r="P6" t="inlineStr">
+      <c r="S6" t="inlineStr">
         <is>
           <t>reject</t>
         </is>
       </c>
-      <c r="Q6" t="inlineStr">
+      <c r="T6" t="inlineStr">
         <is>
           <t>critical</t>
         </is>
       </c>
-      <c r="R6" t="inlineStr">
+      <c r="U6" t="inlineStr">
         <is>
           <t>strict_full_match_required:none</t>
         </is>

</xml_diff>

<commit_message>
Make small tender XLSX source URL columns clickable
</commit_message>
<xml_diff>
--- a/exports/small_tender_report_auction_prod.xlsx
+++ b/exports/small_tender_report_auction_prod.xlsx
@@ -17,12 +17,19 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <color theme="10"/>
+      <sz val="12"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -43,14 +50,17 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8" hidden="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -537,7 +547,7 @@
       <c r="C2" t="n">
         <v>2790</v>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" s="1" t="inlineStr">
         <is>
           <t>https://zakupki.mos.ru/auction/10208353</t>
         </is>
@@ -578,7 +588,7 @@
       <c r="N2" t="n">
         <v>3485</v>
       </c>
-      <c r="O2" t="inlineStr">
+      <c r="O2" s="1" t="inlineStr">
         <is>
           <t>https://zakupki.mos.ru/auction/10208353</t>
         </is>
@@ -590,7 +600,7 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>auction_api_costPerUnit</t>
+          <t>from_input</t>
         </is>
       </c>
       <c r="R2" t="n">
@@ -626,7 +636,7 @@
       <c r="C3" t="n">
         <v>2790</v>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D3" s="1" t="inlineStr">
         <is>
           <t>https://zakupki.mos.ru/auction/10208353</t>
         </is>
@@ -667,7 +677,7 @@
       <c r="N3" t="n">
         <v>2985</v>
       </c>
-      <c r="O3" t="inlineStr">
+      <c r="O3" s="1" t="inlineStr">
         <is>
           <t>https://zakupki.mos.ru/auction/10208353</t>
         </is>
@@ -679,7 +689,7 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>auction_api_costPerUnit</t>
+          <t>from_input</t>
         </is>
       </c>
       <c r="R3" t="n">
@@ -715,7 +725,7 @@
       <c r="C4" t="n">
         <v>2790</v>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D4" s="1" t="inlineStr">
         <is>
           <t>https://zakupki.mos.ru/auction/10208353</t>
         </is>
@@ -756,7 +766,7 @@
       <c r="N4" t="n">
         <v>2790</v>
       </c>
-      <c r="O4" t="inlineStr">
+      <c r="O4" s="1" t="inlineStr">
         <is>
           <t>https://zakupki.mos.ru/auction/10208353</t>
         </is>
@@ -768,7 +778,7 @@
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>auction_api_costPerUnit</t>
+          <t>from_input</t>
         </is>
       </c>
       <c r="R4" t="n">
@@ -804,7 +814,7 @@
       <c r="C5" t="n">
         <v>320</v>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D5" s="1" t="inlineStr">
         <is>
           <t>https://zakupki.mos.ru/auction/10208351</t>
         </is>
@@ -845,7 +855,7 @@
       <c r="N5" t="n">
         <v>320</v>
       </c>
-      <c r="O5" t="inlineStr">
+      <c r="O5" s="1" t="inlineStr">
         <is>
           <t>https://zakupki.mos.ru/auction/10208351</t>
         </is>
@@ -857,7 +867,7 @@
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>auction_api_costPerUnit</t>
+          <t>from_input</t>
         </is>
       </c>
       <c r="R5" t="n">
@@ -893,7 +903,7 @@
       <c r="C6" t="n">
         <v>320</v>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D6" s="1" t="inlineStr">
         <is>
           <t>https://zakupki.mos.ru/auction/10208351</t>
         </is>
@@ -934,7 +944,7 @@
       <c r="N6" t="n">
         <v>3500</v>
       </c>
-      <c r="O6" t="inlineStr">
+      <c r="O6" s="1" t="inlineStr">
         <is>
           <t>https://zakupki.mos.ru/auction/10208351</t>
         </is>
@@ -946,7 +956,7 @@
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>auction_api_costPerUnit</t>
+          <t>from_input</t>
         </is>
       </c>
       <c r="R6" t="n">
@@ -969,6 +979,18 @@
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O2" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O3" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D4" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O4" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D5" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O5" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D6" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O6" r:id="rId10"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
small-tender: forbid zakupki domains as market price sources
</commit_message>
<xml_diff>
--- a/exports/small_tender_report_auction_prod.xlsx
+++ b/exports/small_tender_report_auction_prod.xlsx
@@ -552,9 +552,6 @@
           <t>https://zakupki.mos.ru/auction/10208353</t>
         </is>
       </c>
-      <c r="E2" t="n">
-        <v>3485</v>
-      </c>
       <c r="F2" t="inlineStr">
         <is>
           <t>2026-05-22T07:27:55.695031+00:00</t>
@@ -585,9 +582,6 @@
       <c r="M2" t="b">
         <v>0</v>
       </c>
-      <c r="N2" t="n">
-        <v>3485</v>
-      </c>
       <c r="O2" s="1" t="inlineStr">
         <is>
           <t>https://zakupki.mos.ru/auction/10208353</t>
@@ -600,11 +594,8 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>from_input</t>
-        </is>
-      </c>
-      <c r="R2" t="n">
-        <v>-24.91</v>
+          <t>invalid_market_source_domain</t>
+        </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
@@ -641,9 +632,6 @@
           <t>https://zakupki.mos.ru/auction/10208353</t>
         </is>
       </c>
-      <c r="E3" t="n">
-        <v>2985</v>
-      </c>
       <c r="F3" t="inlineStr">
         <is>
           <t>2026-05-22T07:27:55.695031+00:00</t>
@@ -674,9 +662,6 @@
       <c r="M3" t="b">
         <v>0</v>
       </c>
-      <c r="N3" t="n">
-        <v>2985</v>
-      </c>
       <c r="O3" s="1" t="inlineStr">
         <is>
           <t>https://zakupki.mos.ru/auction/10208353</t>
@@ -689,11 +674,8 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>from_input</t>
-        </is>
-      </c>
-      <c r="R3" t="n">
-        <v>-6.99</v>
+          <t>invalid_market_source_domain</t>
+        </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
@@ -730,9 +712,6 @@
           <t>https://zakupki.mos.ru/auction/10208353</t>
         </is>
       </c>
-      <c r="E4" t="n">
-        <v>2790</v>
-      </c>
       <c r="F4" t="inlineStr">
         <is>
           <t>2026-05-22T07:27:55.695031+00:00</t>
@@ -763,9 +742,6 @@
       <c r="M4" t="b">
         <v>0</v>
       </c>
-      <c r="N4" t="n">
-        <v>2790</v>
-      </c>
       <c r="O4" s="1" t="inlineStr">
         <is>
           <t>https://zakupki.mos.ru/auction/10208353</t>
@@ -778,11 +754,8 @@
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>from_input</t>
-        </is>
-      </c>
-      <c r="R4" t="n">
-        <v>0</v>
+          <t>invalid_market_source_domain</t>
+        </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
@@ -819,9 +792,6 @@
           <t>https://zakupki.mos.ru/auction/10208351</t>
         </is>
       </c>
-      <c r="E5" t="n">
-        <v>320</v>
-      </c>
       <c r="F5" t="inlineStr">
         <is>
           <t>2026-05-22T07:27:55.695031+00:00</t>
@@ -852,9 +822,6 @@
       <c r="M5" t="b">
         <v>0</v>
       </c>
-      <c r="N5" t="n">
-        <v>320</v>
-      </c>
       <c r="O5" s="1" t="inlineStr">
         <is>
           <t>https://zakupki.mos.ru/auction/10208351</t>
@@ -867,11 +834,8 @@
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>from_input</t>
-        </is>
-      </c>
-      <c r="R5" t="n">
-        <v>0</v>
+          <t>invalid_market_source_domain</t>
+        </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
@@ -908,9 +872,6 @@
           <t>https://zakupki.mos.ru/auction/10208351</t>
         </is>
       </c>
-      <c r="E6" t="n">
-        <v>3500</v>
-      </c>
       <c r="F6" t="inlineStr">
         <is>
           <t>2026-05-22T07:27:55.695031+00:00</t>
@@ -941,9 +902,6 @@
       <c r="M6" t="b">
         <v>0</v>
       </c>
-      <c r="N6" t="n">
-        <v>3500</v>
-      </c>
       <c r="O6" s="1" t="inlineStr">
         <is>
           <t>https://zakupki.mos.ru/auction/10208351</t>
@@ -956,11 +914,8 @@
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>from_input</t>
-        </is>
-      </c>
-      <c r="R6" t="n">
-        <v>-993.75</v>
+          <t>invalid_market_source_domain</t>
+        </is>
       </c>
       <c r="S6" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Use external market sources for auction prod report
</commit_message>
<xml_diff>
--- a/exports/small_tender_report_auction_prod.xlsx
+++ b/exports/small_tender_report_auction_prod.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U6"/>
+  <dimension ref="A1:V6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -454,80 +454,85 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
+          <t>found_offer_unit_price</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>source_domain</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
           <t>collected_at</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>tz_extraction_status</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>tz_extraction_reason</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>tz_attachment_path</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>tz_text_len</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>tz_match_type</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>tz_overlap_ratio</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>strict_full_match</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>found_offer_unit_price</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>market_price_source_url</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>market_price_source_domain</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>market_price_source_note</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>margin_pct</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>decision_status</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>risk_level</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>decision_reason</t>
         </is>
@@ -549,67 +554,81 @@
       </c>
       <c r="D2" s="1" t="inlineStr">
         <is>
-          <t>https://zakupki.mos.ru/auction/10208353</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>2026-05-22T07:27:55.695031+00:00</t>
-        </is>
+          <t>https://standonline.ru/catalog/stendy_po_tematikam/grazhdanskaya_oborona/9002/</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>1823</v>
+      </c>
+      <c r="F2" t="n">
+        <v>1823</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr"/>
+          <t>standonline.ru</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>2026-05-22T09:26:34Z</t>
+        </is>
+      </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>exports/tz_files_auction/10208353/Техническое задание.docx</t>
-        </is>
-      </c>
-      <c r="J2" t="n">
-        <v>18272</v>
-      </c>
-      <c r="K2" t="inlineStr">
+          <t>failed</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>no_attachment_manifest_entry</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M2" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="L2" t="n">
-        <v>0.0065</v>
-      </c>
-      <c r="M2" t="b">
-        <v>0</v>
-      </c>
-      <c r="O2" s="1" t="inlineStr">
-        <is>
-          <t>https://zakupki.mos.ru/auction/10208353</t>
-        </is>
-      </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>zakupki.mos.ru</t>
+      <c r="N2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O2" t="b">
+        <v>0</v>
+      </c>
+      <c r="P2" s="1" t="inlineStr">
+        <is>
+          <t>https://standonline.ru/catalog/stendy_po_tematikam/grazhdanskaya_oborona/9002/</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>invalid_market_source_domain</t>
-        </is>
-      </c>
-      <c r="S2" t="inlineStr">
+          <t>standonline.ru</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>from_input</t>
+        </is>
+      </c>
+      <c r="S2" t="n">
+        <v>34.66</v>
+      </c>
+      <c r="T2" t="inlineStr">
         <is>
           <t>reject</t>
         </is>
       </c>
-      <c r="T2" t="inlineStr">
+      <c r="U2" t="inlineStr">
         <is>
           <t>critical</t>
         </is>
       </c>
-      <c r="U2" t="inlineStr">
-        <is>
-          <t>strict_full_match_required:none</t>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>tz_extraction_failed:no_attachment_manifest_entry</t>
         </is>
       </c>
     </row>
@@ -621,7 +640,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Стенд информационный   ProfMarker " "Пожарная безопасность" , красный, 900х740 мм., 1 карман А4</t>
+          <t>Стенд информационный   ProfMarker "Пожарная безопасность" , красный, 900х740 мм., 1 карман А4</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -629,67 +648,81 @@
       </c>
       <c r="D3" s="1" t="inlineStr">
         <is>
-          <t>https://zakupki.mos.ru/auction/10208353</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>2026-05-22T07:27:55.695031+00:00</t>
-        </is>
+          <t>https://standonline.ru/catalog/stendy_po_tematikam/pozharnaya_bezopasnost/8113/</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>1823</v>
+      </c>
+      <c r="F3" t="n">
+        <v>1823</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr"/>
+          <t>standonline.ru</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>2026-05-22T09:26:34Z</t>
+        </is>
+      </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>exports/tz_files_auction/10208353/Техническое задание.docx</t>
-        </is>
-      </c>
-      <c r="J3" t="n">
-        <v>18272</v>
-      </c>
-      <c r="K3" t="inlineStr">
+          <t>failed</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>no_attachment_manifest_entry</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M3" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="L3" t="n">
-        <v>0.0104</v>
-      </c>
-      <c r="M3" t="b">
-        <v>0</v>
-      </c>
-      <c r="O3" s="1" t="inlineStr">
-        <is>
-          <t>https://zakupki.mos.ru/auction/10208353</t>
-        </is>
-      </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>zakupki.mos.ru</t>
+      <c r="N3" t="n">
+        <v>0</v>
+      </c>
+      <c r="O3" t="b">
+        <v>0</v>
+      </c>
+      <c r="P3" s="1" t="inlineStr">
+        <is>
+          <t>https://standonline.ru/catalog/stendy_po_tematikam/pozharnaya_bezopasnost/8113/</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>invalid_market_source_domain</t>
-        </is>
-      </c>
-      <c r="S3" t="inlineStr">
+          <t>standonline.ru</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>from_input</t>
+        </is>
+      </c>
+      <c r="S3" t="n">
+        <v>34.66</v>
+      </c>
+      <c r="T3" t="inlineStr">
         <is>
           <t>reject</t>
         </is>
       </c>
-      <c r="T3" t="inlineStr">
+      <c r="U3" t="inlineStr">
         <is>
           <t>critical</t>
         </is>
       </c>
-      <c r="U3" t="inlineStr">
-        <is>
-          <t>strict_full_match_required:none</t>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>tz_extraction_failed:no_attachment_manifest_entry</t>
         </is>
       </c>
     </row>
@@ -709,67 +742,81 @@
       </c>
       <c r="D4" s="1" t="inlineStr">
         <is>
-          <t>https://zakupki.mos.ru/auction/10208353</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>2026-05-22T07:27:55.695031+00:00</t>
-        </is>
+          <t>https://standonline.ru/catalog/stendy_dlya_organizatsiy/vooruzhennye_sily/13774/</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>2916</v>
+      </c>
+      <c r="F4" t="n">
+        <v>2916</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr"/>
+          <t>standonline.ru</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>2026-05-22T09:26:34Z</t>
+        </is>
+      </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>exports/tz_files_auction/10208353/Техническое задание.docx</t>
-        </is>
-      </c>
-      <c r="J4" t="n">
-        <v>18272</v>
-      </c>
-      <c r="K4" t="inlineStr">
+          <t>failed</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>no_attachment_manifest_entry</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M4" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="L4" t="n">
-        <v>0.0091</v>
-      </c>
-      <c r="M4" t="b">
-        <v>0</v>
-      </c>
-      <c r="O4" s="1" t="inlineStr">
-        <is>
-          <t>https://zakupki.mos.ru/auction/10208353</t>
-        </is>
-      </c>
-      <c r="P4" t="inlineStr">
-        <is>
-          <t>zakupki.mos.ru</t>
+      <c r="N4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O4" t="b">
+        <v>0</v>
+      </c>
+      <c r="P4" s="1" t="inlineStr">
+        <is>
+          <t>https://standonline.ru/catalog/stendy_dlya_organizatsiy/vooruzhennye_sily/13774/</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>invalid_market_source_domain</t>
-        </is>
-      </c>
-      <c r="S4" t="inlineStr">
+          <t>standonline.ru</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>from_input</t>
+        </is>
+      </c>
+      <c r="S4" t="n">
+        <v>-4.52</v>
+      </c>
+      <c r="T4" t="inlineStr">
         <is>
           <t>reject</t>
         </is>
       </c>
-      <c r="T4" t="inlineStr">
+      <c r="U4" t="inlineStr">
         <is>
           <t>critical</t>
         </is>
       </c>
-      <c r="U4" t="inlineStr">
-        <is>
-          <t>strict_full_match_required:none</t>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>tz_extraction_failed:no_attachment_manifest_entry</t>
         </is>
       </c>
     </row>
@@ -789,67 +836,81 @@
       </c>
       <c r="D5" s="1" t="inlineStr">
         <is>
-          <t>https://zakupki.mos.ru/auction/10208351</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>2026-05-22T07:27:55.695031+00:00</t>
-        </is>
+          <t>https://lider-ic.ru/shop/armature-sip-of-04-1-kv/junction-clamps-04-1-kv/sealed-junction-clamps-04-1-kv/sealed-junction-clamps-for-insulated-conductors-of-04-1-kv/sliw50-piercing-clamp-alcu-10-50-mm2-alcu-15-10-mm2-sealed/</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>209</v>
+      </c>
+      <c r="F5" t="n">
+        <v>209</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr"/>
+          <t>lider-ic.ru</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>2026-05-22T09:26:34Z</t>
+        </is>
+      </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>exports/tz_files_auction/10208351/Приложение №1 к Договору (Техническое задание).docx</t>
-        </is>
-      </c>
-      <c r="J5" t="n">
-        <v>13281</v>
-      </c>
-      <c r="K5" t="inlineStr">
+          <t>failed</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>no_attachment_manifest_entry</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M5" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="L5" t="n">
-        <v>0.0059</v>
-      </c>
-      <c r="M5" t="b">
-        <v>0</v>
-      </c>
-      <c r="O5" s="1" t="inlineStr">
-        <is>
-          <t>https://zakupki.mos.ru/auction/10208351</t>
-        </is>
-      </c>
-      <c r="P5" t="inlineStr">
-        <is>
-          <t>zakupki.mos.ru</t>
+      <c r="N5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O5" t="b">
+        <v>0</v>
+      </c>
+      <c r="P5" s="1" t="inlineStr">
+        <is>
+          <t>https://lider-ic.ru/shop/armature-sip-of-04-1-kv/junction-clamps-04-1-kv/sealed-junction-clamps-04-1-kv/sealed-junction-clamps-for-insulated-conductors-of-04-1-kv/sliw50-piercing-clamp-alcu-10-50-mm2-alcu-15-10-mm2-sealed/</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>invalid_market_source_domain</t>
-        </is>
-      </c>
-      <c r="S5" t="inlineStr">
+          <t>lider-ic.ru</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>from_input</t>
+        </is>
+      </c>
+      <c r="S5" t="n">
+        <v>34.69</v>
+      </c>
+      <c r="T5" t="inlineStr">
         <is>
           <t>reject</t>
         </is>
       </c>
-      <c r="T5" t="inlineStr">
+      <c r="U5" t="inlineStr">
         <is>
           <t>critical</t>
         </is>
       </c>
-      <c r="U5" t="inlineStr">
-        <is>
-          <t>strict_full_match_required:none</t>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>tz_extraction_failed:no_attachment_manifest_entry</t>
         </is>
       </c>
     </row>
@@ -869,82 +930,96 @@
       </c>
       <c r="D6" s="1" t="inlineStr">
         <is>
-          <t>https://zakupki.mos.ru/auction/10208351</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>2026-05-22T07:27:55.695031+00:00</t>
-        </is>
+          <t>https://ekf.market/catalog/products/plc-jxb-10-35gy/</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>67</v>
+      </c>
+      <c r="F6" t="n">
+        <v>67</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr"/>
+          <t>ekf.market</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>2026-05-22T09:26:34Z</t>
+        </is>
+      </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>exports/tz_files_auction/10208351/Приложение №1 к Договору (Техническое задание).docx</t>
-        </is>
-      </c>
-      <c r="J6" t="n">
-        <v>13281</v>
-      </c>
-      <c r="K6" t="inlineStr">
+          <t>failed</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>no_attachment_manifest_entry</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="n">
+        <v>0</v>
+      </c>
+      <c r="M6" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="L6" t="n">
-        <v>0</v>
-      </c>
-      <c r="M6" t="b">
-        <v>0</v>
-      </c>
-      <c r="O6" s="1" t="inlineStr">
-        <is>
-          <t>https://zakupki.mos.ru/auction/10208351</t>
-        </is>
-      </c>
-      <c r="P6" t="inlineStr">
-        <is>
-          <t>zakupki.mos.ru</t>
+      <c r="N6" t="n">
+        <v>0</v>
+      </c>
+      <c r="O6" t="b">
+        <v>0</v>
+      </c>
+      <c r="P6" s="1" t="inlineStr">
+        <is>
+          <t>https://ekf.market/catalog/products/plc-jxb-10-35gy/</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>invalid_market_source_domain</t>
-        </is>
-      </c>
-      <c r="S6" t="inlineStr">
+          <t>ekf.market</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>from_input</t>
+        </is>
+      </c>
+      <c r="S6" t="n">
+        <v>79.06</v>
+      </c>
+      <c r="T6" t="inlineStr">
         <is>
           <t>reject</t>
         </is>
       </c>
-      <c r="T6" t="inlineStr">
+      <c r="U6" t="inlineStr">
         <is>
           <t>critical</t>
         </is>
       </c>
-      <c r="U6" t="inlineStr">
-        <is>
-          <t>strict_full_match_required:none</t>
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>tz_extraction_failed:no_attachment_manifest_entry</t>
         </is>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O2" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P2" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O3" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P3" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D4" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O4" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P4" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D5" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O5" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P5" r:id="rId8"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D6" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O6" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P6" r:id="rId10"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>